<commit_message>
docs: restamp e2e-matrix and VP deck census after F-070
Offline POSIX driver --hypothesis-profile ci (31 PASS). suite:root 3123,
backend-validation 357. Committed matrix is NOT-RUN for Tier D, not SKIP.
VP_DECK/DECK_A_PLUS census is 68 done + 2 deferred of 70. Discrimination
n=60 re-measured with unchanged means. eval_metrics.json 0-10s not retuned.

Co-authored-by: Ian Cruickshank <ianshank@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/e2e-matrix/e2e-test-matrix.xlsx
+++ b/docs/e2e-matrix/e2e-test-matrix.xlsx
@@ -575,7 +575,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>35404</t>
+          <t>32766</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>23540</t>
+          <t>23435</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2052</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>7285</t>
+          <t>5247</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>517</t>
+          <t>497</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -910,17 +910,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2978 tests</t>
+          <t>3123 tests</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>70737</t>
+          <t>76508</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2978</t>
+          <t>3123</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>28</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -978,17 +978,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2978 tests</t>
+          <t>3123 tests</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>71836</t>
+          <t>76276</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2978</t>
+          <t>3123</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>28</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1047,7 +1047,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>20417</t>
+          <t>20589</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -1095,7 +1095,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>631</t>
+          <t>660</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -1143,7 +1143,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>58</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -1191,7 +1191,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>89</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -1239,7 +1239,7 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>88</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -1287,7 +1287,7 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>718</t>
+          <t>709</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -1375,7 +1375,7 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>88</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -1471,7 +1471,7 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>383</t>
+          <t>397</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -1519,7 +1519,7 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>375</t>
+          <t>384</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -1567,7 +1567,7 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>384</t>
+          <t>387</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
@@ -1615,7 +1615,7 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>375</t>
+          <t>383</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -1663,7 +1663,7 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>411</t>
+          <t>416</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -1711,7 +1711,7 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>398</t>
+          <t>409</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>88</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -1811,7 +1811,7 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>97</t>
+          <t>99</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -1995,7 +1995,7 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>54</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -2043,7 +2043,7 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>107</t>
+          <t>110</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>355 tests</t>
+          <t>357 tests</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>355</t>
+          <t>357</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>4474</t>
+          <t>4451</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2972,7 +2972,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>355</t>
+          <t>357</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2978</t>
+          <t>3123</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2978</t>
+          <t>3123</t>
         </is>
       </c>
     </row>
@@ -3315,7 +3315,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>27e5b8cb588569f021e8bc83b7592fa67be91015</t>
+          <t>f83f7f071435b04cb4926848b147cdfd7a381588</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>cursor/e2e-matrix-restamp-24d8</t>
+          <t>cursor/e2e-vp-capture-eefa</t>
         </is>
       </c>
     </row>
@@ -3339,7 +3339,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-09T01:57:55+00:00</t>
+          <t>2026-09-15T01:17:11+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(ci): regenerate e2e-matrix from offline nightly report
Nightly e2e-freshness failed because docs/e2e-matrix/e2e-matrix.md was
stale against artifacts/e2e-report (PASS 31). Regenerated with
`python tests/test_e2e_matrix.py --update` from the latest offline driver
artifact; no runner or test-logic changes.
</commit_message>
<xml_diff>
--- a/docs/e2e-matrix/e2e-test-matrix.xlsx
+++ b/docs/e2e-matrix/e2e-test-matrix.xlsx
@@ -575,7 +575,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>32766</t>
+          <t>55192</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>23435</t>
+          <t>36398</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>3794</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>5247</t>
+          <t>11974</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>497</t>
+          <t>838</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -910,17 +910,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>3123 tests</t>
+          <t>3184 tests</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>76508</t>
+          <t>111833</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>3123</t>
+          <t>3184</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>36</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -978,17 +978,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>3123 tests</t>
+          <t>3184 tests</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>76276</t>
+          <t>102260</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>3123</t>
+          <t>3184</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>36</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1047,7 +1047,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>20589</t>
+          <t>31742</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -1095,7 +1095,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>660</t>
+          <t>933</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -1143,7 +1143,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>90</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -1191,7 +1191,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>142</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -1239,7 +1239,7 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>143</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -1287,7 +1287,7 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>709</t>
+          <t>1330</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -1375,7 +1375,7 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>143</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -1423,7 +1423,7 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>144</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1471,7 +1471,7 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>397</t>
+          <t>550</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -1519,7 +1519,7 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>384</t>
+          <t>547</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -1567,7 +1567,7 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>387</t>
+          <t>558</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
@@ -1615,7 +1615,7 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>383</t>
+          <t>530</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -1663,7 +1663,7 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>416</t>
+          <t>568</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -1711,7 +1711,7 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>605</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>139</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
@@ -1811,7 +1811,7 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>155</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -1859,7 +1859,7 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>136</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
@@ -1907,7 +1907,7 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>146</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -1995,7 +1995,7 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>85</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -2043,7 +2043,7 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>177</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -2163,7 +2163,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>4451</t>
+          <t>7905</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>3123</t>
+          <t>3184</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3123</t>
+          <t>3184</t>
         </is>
       </c>
     </row>
@@ -3315,7 +3315,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>f83f7f071435b04cb4926848b147cdfd7a381588</t>
+          <t>5cf4758eae0913a1f1afefb14a65cc9ba3897eeb</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>cursor/e2e-vp-capture-eefa</t>
+          <t>main</t>
         </is>
       </c>
     </row>
@@ -3339,7 +3339,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-15T01:17:11+00:00</t>
+          <t>2026-09-20T13:50:01+00:00</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Linux-6.12.94+-x86_64-with-glibc2.39</t>
+          <t>Linux-6.12.94+-x86_64-with-glibc2.41</t>
         </is>
       </c>
     </row>
@@ -3363,7 +3363,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3.12.3</t>
+          <t>3.13.5</t>
         </is>
       </c>
     </row>

</xml_diff>